<commit_message>
Final Commit For The Day
</commit_message>
<xml_diff>
--- a/output/BIFM_UT_Processing_Report.xlsx
+++ b/output/BIFM_UT_Processing_Report.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>NNELO TAUNYANE</t>
+          <t>NNelo Taunyane</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>NNELO TAUNYANE</t>
+          <t>NNelo Taunyane</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>2026-07-02T16:37:07</t>
+          <t>2026-07-02T17:01:41</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>NNELO TAUNYANE</t>
+          <t>NNelo Taunyane</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-02T16:37:07</t>
+          <t>2026-07-02T17:01:41</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>NNELO TAUNYANE</t>
+          <t>NNelo Taunyane</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="P6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02T16:37:07</t>
+          <t>2026-07-02T17:01:41</t>
         </is>
       </c>
       <c r="Q6" s="4" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>NNELO TAUNYANE</t>
+          <t>NNelo Taunyane</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="P8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02T16:37:07</t>
+          <t>2026-07-02T17:01:41</t>
         </is>
       </c>
       <c r="Q8" s="4" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>NNELO TAUNYANE</t>
+          <t>NNelo Taunyane</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr"/>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="P10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02T16:37:07</t>
+          <t>2026-07-02T17:01:41</t>
         </is>
       </c>
       <c r="Q10" s="4" t="inlineStr">
@@ -2403,7 +2403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2684,37 +2684,37 @@
       <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>GSGF - NNELO TAUNYANE</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>DIS_GSG</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>id_expiry_date</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>ID expiry date not captured</t>
-        </is>
-      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>nnelo@bifm.co.bw</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2734,12 +2734,12 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>contact_number</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>nnelo@bifm.co.bw</t>
+          <t>71234567</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -2767,12 +2767,12 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>contact_number</t>
+          <t>branch_code</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>71234567</t>
+          <t>064967</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -2800,12 +2800,12 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>branch_code</t>
+          <t>fund_category</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>064967</t>
+          <t>Non-Money Market (GSGF)</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -2816,140 +2816,140 @@
       <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>GSGF - NNELO TAUNYANE</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>DIS_GSG</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>fund_category</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Non-Money Market (GSGF)</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>instruction_mode</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Could not determine instruction mode - no closure tick, percentage, or withdrawal/deposit amount was found</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>DIS - NNELO</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>fund_name</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Mandatory field missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>DIS - NNELO</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>nnelo@bifm.co.bw</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>GSGF - NNELO TAUNYANE</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>DIS_GSG</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>instruction_mode</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Could not determine instruction mode - no closure tick, percentage, or withdrawal/deposit amount was found</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>DIS - NNELO</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>DIS</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>fund_name</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Mandatory field missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>DIS - NNELO</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>DIS</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>id_expiry_date</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>ID expiry date not captured</t>
-        </is>
-      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>contact_number</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>71234567</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -2969,12 +2969,12 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>branch_code</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>nnelo@bifm.co.bw</t>
+          <t>064967</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -2985,70 +2985,74 @@
       <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>DIS - NNELO</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>DIS</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>contact_number</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>71234567</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>fund_number</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Field is blank</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>DIS - NNELO</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>DIS</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>branch_code</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>064967</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>fund_category</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Unknown - Fund Name Not Extracted</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Fund category could not be determined - fund name unclear</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -3068,395 +3072,391 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
+          <t>instruction_mode</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Could not determine instruction mode - no closure tick, percentage, or withdrawal/deposit amount was found</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>DEBIT - NNELO</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>DEBIT</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>instruction_type</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Mandatory field missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>DEBIT - NNELO</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>DEBIT</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>nnelo@bifm.co.bw</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>DEBIT - NNELO</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>DEBIT</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>contact_number</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>71234567</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>DEBIT - NNELO</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>DEBIT</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>branch_code</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>064967</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>DEBIT - NNELO</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>DEBIT</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
           <t>fund_number</t>
         </is>
       </c>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>WARNING</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Field is blank</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>DIS - NNELO</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>DIS</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>DEBIT - NNELO</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>DEBIT</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>fund_category</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>Unknown - Fund Name Not Extracted</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>WARNING</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Fund category could not be determined - fund name unclear</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>DIS - NNELO</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>DIS</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>instruction_mode</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Could not determine instruction mode - no closure tick, percentage, or withdrawal/deposit amount was found</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>ADD - NNELO</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>fund_name</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Mandatory field missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>DEBIT - NNELO</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>DEBIT</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>instruction_type</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>ADD - NNELO</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>fund_number</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>Mandatory field missing</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>DEBIT - NNELO</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>DEBIT</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>id_expiry_date</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>ID expiry date not captured</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>ADD - NNELO</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>nnelo@bifm.co.bw</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>DEBIT - NNELO</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>DEBIT</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>nnelo@bifm.co.bw</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>ADD - NNELO</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>contact_number</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>71234567</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>DEBIT - NNELO</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>DEBIT</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>contact_number</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>71234567</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>ADD - NNELO</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>branch_code</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>064967</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>DEBIT - NNELO</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>DEBIT</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>branch_code</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>064967</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>DEBIT - NNELO</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>DEBIT</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>fund_number</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>Field is blank</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>DEBIT - NNELO</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>DEBIT</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>fund_category</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>Unknown - Fund Name Not Extracted</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>Fund category could not be determined - fund name unclear</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>fund_name</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>Mandatory field missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>fund_number</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>Mandatory field missing</t>
-        </is>
-      </c>
+      <c r="G31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>id_expiry_date</t>
+          <t>fund_number</t>
         </is>
       </c>
       <c r="E32" s="3" t="n"/>
@@ -3487,174 +3487,42 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>ID expiry date not captured</t>
+          <t>Field is blank</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>ADD - NNELO</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>ADD</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>nnelo@bifm.co.bw</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>contact_number</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>71234567</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>branch_code</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>064967</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>fund_number</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="n"/>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>fund_category</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Unknown - Fund Name Not Extracted</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>WARNING</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>Field is blank</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>fund_category</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>Unknown - Fund Name Not Extracted</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Fund category could not be determined - fund name unclear</t>
         </is>
@@ -3765,7 +3633,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-02T16:38:17</t>
+          <t>2026-07-02T17:02:48</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3775,7 +3643,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KYC_381234567_TAUNYANE_20260702_1.pdf</t>
+          <t>KYC_381234567_TAUNYANE_20260702_1_2.pdf</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -3804,12 +3672,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-02T16:37:07</t>
+          <t>2026-07-02T17:01:41</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\KYC_381234567_TAUNYANE_20260702_1.pdf</t>
+          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\KYC_381234567_TAUNYANE_20260702_1_2.pdf</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -3827,7 +3695,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-02T16:38:17</t>
+          <t>2026-07-02T17:02:48</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3837,7 +3705,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DIS_GSG_381234567_TAUNYANE_20260702_1.pdf</t>
+          <t>DIS_GSG_381234567_TAUNYANE_20260702_1_2.pdf</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -3866,12 +3734,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-02T16:37:07</t>
+          <t>2026-07-02T17:01:41</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\DIS_GSG_381234567_TAUNYANE_20260702_1.pdf</t>
+          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\DIS_GSG_381234567_TAUNYANE_20260702_1_2.pdf</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -3889,7 +3757,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-02T16:38:17</t>
+          <t>2026-07-02T17:02:48</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3899,7 +3767,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DIS_381234567_TAUNYANE_20260702_VALIDATIONFAILEDFUND_NAME_1.pdf</t>
+          <t>DIS_381234567_TAUNYANE_20260702_VALIDATIONFAILEDFUND_NAME_1_2.pdf</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -3932,12 +3800,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-02T16:37:07</t>
+          <t>2026-07-02T17:01:41</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\Rejected\DIS_381234567_TAUNYANE_20260702_VALIDATIONFAILEDFUND_NAME_1.pdf</t>
+          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\Rejected\DIS_381234567_TAUNYANE_20260702_VALIDATIONFAILEDFUND_NAME_1_2.pdf</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -3955,7 +3823,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-02T16:38:17</t>
+          <t>2026-07-02T17:02:48</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3965,7 +3833,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DEBIT_381234567_TAUNYANE_20260702_VALIDATIONFAILEDINSTRUCTION_TYPE_1.pdf</t>
+          <t>DEBIT_381234567_TAUNYANE_20260702_VALIDATIONFAILEDINSTRUCTION_TYPE_1_2.pdf</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -3998,12 +3866,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-02T16:37:07</t>
+          <t>2026-07-02T17:01:41</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\Rejected\DEBIT_381234567_TAUNYANE_20260702_VALIDATIONFAILEDINSTRUCTION_TYPE_1.pdf</t>
+          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\Rejected\DEBIT_381234567_TAUNYANE_20260702_VALIDATIONFAILEDINSTRUCTION_TYPE_1_2.pdf</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -4021,7 +3889,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-02T16:38:17</t>
+          <t>2026-07-02T17:02:48</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4031,7 +3899,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ADD_381234567_TAUNYANE_20260702_VALIDATIONFAILEDFUND_NAMEFUND_NUMBER_1.pdf</t>
+          <t>ADD_381234567_TAUNYANE_20260702_VALIDATIONFAILEDFUND_NAMEFUND_NUMBER_1_2.pdf</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -4064,12 +3932,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-02T16:37:07</t>
+          <t>2026-07-02T17:01:41</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\Rejected\ADD_381234567_TAUNYANE_20260702_VALIDATIONFAILEDFUND_NAMEFUND_NUMBER_1.pdf</t>
+          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\Rejected\ADD_381234567_TAUNYANE_20260702_VALIDATIONFAILEDFUND_NAMEFUND_NUMBER_1_2.pdf</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">

</xml_diff>

<commit_message>
Final Final Commit of the Day
</commit_message>
<xml_diff>
--- a/output/BIFM_UT_Processing_Report.xlsx
+++ b/output/BIFM_UT_Processing_Report.xlsx
@@ -39,7 +39,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -66,12 +66,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
@@ -89,13 +83,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -694,87 +687,87 @@
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>98% confidence — majority vote: 4/5 documents agree on this value (differs on: GSGF - NNELO TAUNYANE) — value taken from KYC - Nnelo Taunyane</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — 5/5 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>90% confidence — NO MAJORITY — 2-way tie across 4 documents, no value has more support than another (sources: DEBIT - NNELO, DIS - NNELO, GSGF - NNELO TAUNYANE, KYC - Nnelo Taunyane) — best guess shown from KYC - Nnelo Taunyane, needs manual review before relying on this value — value taken from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — majority vote: 3/5 documents agree on this value (differs on: ADD - NNELO, DEBIT - NNELO) — value taken from KYC - Nnelo Taunyane</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — 5/5 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
-        </is>
-      </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
+          <t>98% confidence — 2/2 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
+          <t>98% confidence — 3/3 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
+          <t>90% confidence — NO MAJORITY — 3-way tie across 3 documents, no value has more support than another (sources: DIS - NNELO, GSGF - NNELO TAUNYANE, KYC - Nnelo Taunyane) — best guess shown from KYC - Nnelo Taunyane, needs manual review before relying on this value — value taken from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
+          <t>98% confidence — 3/3 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
+          <t>98% confidence — 3/3 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — 1/1 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
+          <t>98% confidence — 3/3 document(s) agree — value taken from KYC - Nnelo Taunyane</t>
         </is>
       </c>
     </row>
@@ -789,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP11"/>
+  <dimension ref="A1:BB11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -803,14 +796,14 @@
     <col width="45" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
-    <col width="27" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="43" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="27" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
     <col width="21" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
-    <col width="45" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
     <col width="45" customWidth="1" min="20" max="20"/>
     <col width="45" customWidth="1" min="21" max="21"/>
     <col width="45" customWidth="1" min="22" max="22"/>
@@ -834,6 +827,18 @@
     <col width="45" customWidth="1" min="40" max="40"/>
     <col width="45" customWidth="1" min="41" max="41"/>
     <col width="45" customWidth="1" min="42" max="42"/>
+    <col width="45" customWidth="1" min="43" max="43"/>
+    <col width="45" customWidth="1" min="44" max="44"/>
+    <col width="45" customWidth="1" min="45" max="45"/>
+    <col width="45" customWidth="1" min="46" max="46"/>
+    <col width="45" customWidth="1" min="47" max="47"/>
+    <col width="45" customWidth="1" min="48" max="48"/>
+    <col width="45" customWidth="1" min="49" max="49"/>
+    <col width="45" customWidth="1" min="50" max="50"/>
+    <col width="45" customWidth="1" min="51" max="51"/>
+    <col width="45" customWidth="1" min="52" max="52"/>
+    <col width="45" customWidth="1" min="53" max="53"/>
+    <col width="45" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -879,170 +884,230 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>fund_number</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>fund_category</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>processing_cutoff</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>fund_category_priority</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>overall_validation_status</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>instruction_status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>rejection_reason</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>channel</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>upload_date</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>captured_by</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>authorized_by</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>contact_number</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>citizenship</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>bank_account_name</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>bank_name</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>account_number</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>branch_name</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>branch_code</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>account_type_banking</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>account_category</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>account_closure</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>change_amount</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>commencement_date</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>country_of_birth</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>disinvestment_amount</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>employer</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>entity_name</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>income_distribution</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>instruction_mode</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>instruction_type</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>kyc_certified_id</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>kyc_completeness_flag</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>kyc_proof_address</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>kyc_proof_banking</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>kyc_proof_source</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>lump_sum_debit_amount</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>occupation</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>payment_method</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>residential_address</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>source_of_contribution</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>source_of_funds</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>source_of_income</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>sub_instruction_type</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>us_ssn</t>
         </is>
@@ -1051,17 +1116,17 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>GSGF - NNELO TAUNYANE</t>
+          <t>DIS - NNELO</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>DIS_GSG</t>
+          <t>DIS</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Disinvestment Form (GSGF)</t>
+          <t>Disinvestment Form (Standard)</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -1076,242 +1141,286 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>11102222</t>
+          <t>111102222</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>BIFM Global Sustainable Growth Fund</t>
+          <t>Bifm Pula Money Market Fund</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Non-Money Market (GSGF)</t>
+          <t>9876543</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Quarterly - 7th of last month of quarter</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
+          <t>Money Market</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>WARNING</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Captured</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr"/>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr"/>
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-02T17:10:12</t>
-        </is>
-      </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
+          <t>2026-07-02T17:16:15</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
           <t>marvel.ai-local-poc</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr"/>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr"/>
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>71234567</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>nnelo@bifm.co.bw</t>
         </is>
       </c>
-      <c r="U2" s="3" t="inlineStr"/>
-      <c r="V2" s="3" t="inlineStr">
-        <is>
-          <t>NNELO TAUNYANE</t>
-        </is>
-      </c>
+      <c r="V2" s="3" t="inlineStr"/>
       <c r="W2" s="3" t="inlineStr">
         <is>
-          <t>STANBIC</t>
+          <t>NNelo Taunyane</t>
         </is>
       </c>
       <c r="X2" s="3" t="inlineStr">
         <is>
-          <t>9060001231234</t>
+          <t>Stanbic</t>
         </is>
       </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
-          <t>FAIRGROUNDS</t>
+          <t>9066001231243</t>
         </is>
       </c>
       <c r="Z2" s="3" t="inlineStr">
         <is>
+          <t>Fairgrounds</t>
+        </is>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
           <t>064967</t>
         </is>
       </c>
-      <c r="AA2" s="3" t="inlineStr">
+      <c r="AB2" s="3" t="inlineStr">
         <is>
           <t>Current</t>
         </is>
       </c>
-      <c r="AB2" s="3" t="inlineStr"/>
       <c r="AC2" s="3" t="inlineStr"/>
-      <c r="AD2" s="3" t="inlineStr"/>
+      <c r="AD2" s="3" t="b">
+        <v>0</v>
+      </c>
       <c r="AE2" s="3" t="inlineStr"/>
-      <c r="AF2" s="3" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
+      <c r="AF2" s="3" t="inlineStr"/>
       <c r="AG2" s="3" t="inlineStr"/>
-      <c r="AH2" s="3" t="inlineStr"/>
+      <c r="AH2" s="3" t="n">
+        <v>1000</v>
+      </c>
       <c r="AI2" s="3" t="inlineStr"/>
       <c r="AJ2" s="3" t="inlineStr"/>
       <c r="AK2" s="3" t="inlineStr"/>
-      <c r="AL2" s="3" t="inlineStr"/>
+      <c r="AL2" s="3" t="inlineStr">
+        <is>
+          <t>Partial Withdrawal</t>
+        </is>
+      </c>
       <c r="AM2" s="3" t="inlineStr"/>
       <c r="AN2" s="3" t="inlineStr"/>
       <c r="AO2" s="3" t="inlineStr"/>
       <c r="AP2" s="3" t="inlineStr"/>
+      <c r="AQ2" s="3" t="inlineStr"/>
+      <c r="AR2" s="3" t="inlineStr"/>
+      <c r="AS2" s="3" t="inlineStr"/>
+      <c r="AT2" s="3" t="inlineStr"/>
+      <c r="AU2" s="3" t="inlineStr"/>
+      <c r="AV2" s="3" t="inlineStr"/>
+      <c r="AW2" s="3" t="inlineStr"/>
+      <c r="AX2" s="3" t="inlineStr"/>
+      <c r="AY2" s="3" t="inlineStr"/>
+      <c r="AZ2" s="3" t="inlineStr"/>
+      <c r="BA2" s="3" t="inlineStr"/>
+      <c r="BB2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr"/>
       <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE</t>
+          <t>98% confidence — extracted from DIS - NNELO</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE</t>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE</t>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE</t>
+          <t>98% confidence — extracted from DIS - NNELO</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr"/>
+          <t>98% confidence — extracted from DIS - NNELO</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DIS - NNELO</t>
+        </is>
+      </c>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="inlineStr"/>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
+      <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr"/>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr"/>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr"/>
-      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
+        </is>
+      </c>
       <c r="AE3" s="2" t="inlineStr"/>
-      <c r="AF3" s="2" t="inlineStr">
-        <is>
-          <t>0% confidence — extracted from GSGF - NNELO TAUNYANE — ⚠ recommend recheck</t>
-        </is>
-      </c>
+      <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
-      <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DIS - NNELO, p.2</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="inlineStr"/>
       <c r="AK3" s="2" t="inlineStr"/>
-      <c r="AL3" s="2" t="inlineStr"/>
+      <c r="AL3" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DIS - NNELO</t>
+        </is>
+      </c>
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr"/>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr"/>
+      <c r="AQ3" s="2" t="inlineStr"/>
+      <c r="AR3" s="2" t="inlineStr"/>
+      <c r="AS3" s="2" t="inlineStr"/>
+      <c r="AT3" s="2" t="inlineStr"/>
+      <c r="AU3" s="2" t="inlineStr"/>
+      <c r="AV3" s="2" t="inlineStr"/>
+      <c r="AW3" s="2" t="inlineStr"/>
+      <c r="AX3" s="2" t="inlineStr"/>
+      <c r="AY3" s="2" t="inlineStr"/>
+      <c r="AZ3" s="2" t="inlineStr"/>
+      <c r="BA3" s="2" t="inlineStr"/>
+      <c r="BB3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>KYC - Nnelo Taunyane</t>
+          <t>DEBIT - NNELO</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>KYC</t>
+          <t>DEBIT</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>KYC (Know Your Customer)</t>
+          <t>Debit Order Form</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1321,7 +1430,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>NNelo Taunyane</t>
+          <t>NNELO TAUNYANE</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1329,957 +1438,1077 @@
           <t>11102222</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>01/02/2003</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Bifm Pula Money Market Fund</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>9876543</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Money Market</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>WARNING</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Captured</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr"/>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-02T17:10:12</t>
-        </is>
-      </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
+          <t>2026-07-02T17:16:15</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
           <t>marvel.ai-local-poc</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr"/>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="S4" s="3" t="inlineStr"/>
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>71234567</t>
         </is>
       </c>
-      <c r="T4" s="3" t="inlineStr">
-        <is>
-          <t>nnelo@bifm.co.bw</t>
-        </is>
-      </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>MOTSWANA</t>
-        </is>
-      </c>
-      <c r="V4" s="3" t="inlineStr">
+          <t>taunyane@bifm.co.bw</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr"/>
+      <c r="W4" s="3" t="inlineStr">
         <is>
           <t>NNELO TAUNYANE</t>
         </is>
       </c>
-      <c r="W4" s="3" t="inlineStr">
+      <c r="X4" s="3" t="inlineStr">
         <is>
           <t>STANBIC</t>
         </is>
       </c>
-      <c r="X4" s="3" t="inlineStr">
-        <is>
-          <t>9060001231234</t>
-        </is>
-      </c>
-      <c r="Y4" s="3" t="inlineStr">
+      <c r="Y4" s="3" t="inlineStr"/>
+      <c r="Z4" s="3" t="inlineStr">
         <is>
           <t>FAIRGROUNDS</t>
         </is>
       </c>
-      <c r="Z4" s="3" t="inlineStr">
+      <c r="AA4" s="3" t="inlineStr">
         <is>
           <t>064967</t>
         </is>
       </c>
-      <c r="AA4" s="3" t="inlineStr">
+      <c r="AB4" s="3" t="inlineStr">
         <is>
           <t>Current</t>
         </is>
       </c>
-      <c r="AB4" s="3" t="inlineStr">
-        <is>
-          <t>Individual</t>
-        </is>
-      </c>
-      <c r="AC4" s="3" t="inlineStr">
-        <is>
-          <t>BOTSWANA</t>
-        </is>
-      </c>
-      <c r="AD4" s="3" t="inlineStr">
-        <is>
-          <t>BIFM UNIT TRUSTS</t>
-        </is>
-      </c>
+      <c r="AC4" s="3" t="inlineStr"/>
+      <c r="AD4" s="3" t="inlineStr"/>
       <c r="AE4" s="3" t="inlineStr">
         <is>
-          <t>NNELO TAUNYANE</t>
-        </is>
-      </c>
-      <c r="AF4" s="3" t="inlineStr"/>
-      <c r="AG4" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH4" s="3" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="AI4" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ4" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK4" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL4" s="3" t="inlineStr">
-        <is>
-          <t>INTERN</t>
-        </is>
-      </c>
+          <t>1000-00</t>
+        </is>
+      </c>
+      <c r="AF4" s="3" t="inlineStr">
+        <is>
+          <t>M 03 Y 2026</t>
+        </is>
+      </c>
+      <c r="AG4" s="3" t="inlineStr"/>
+      <c r="AH4" s="3" t="inlineStr"/>
+      <c r="AI4" s="3" t="inlineStr"/>
+      <c r="AJ4" s="3" t="inlineStr"/>
+      <c r="AK4" s="3" t="inlineStr"/>
+      <c r="AL4" s="3" t="inlineStr"/>
       <c r="AM4" s="3" t="inlineStr">
         <is>
-          <t>PLOT 1234 GABORONE</t>
-        </is>
-      </c>
-      <c r="AN4" s="3" t="inlineStr">
+          <t>Change existing debit order</t>
+        </is>
+      </c>
+      <c r="AN4" s="3" t="inlineStr"/>
+      <c r="AO4" s="3" t="inlineStr"/>
+      <c r="AP4" s="3" t="inlineStr"/>
+      <c r="AQ4" s="3" t="inlineStr"/>
+      <c r="AR4" s="3" t="inlineStr"/>
+      <c r="AS4" s="3" t="inlineStr"/>
+      <c r="AT4" s="3" t="inlineStr"/>
+      <c r="AU4" s="3" t="inlineStr"/>
+      <c r="AV4" s="3" t="inlineStr"/>
+      <c r="AW4" s="3" t="inlineStr">
         <is>
           <t>Salary</t>
         </is>
       </c>
-      <c r="AO4" s="3" t="inlineStr">
-        <is>
-          <t>Ms</t>
-        </is>
-      </c>
-      <c r="AP4" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="AX4" s="3" t="inlineStr"/>
+      <c r="AY4" s="3" t="inlineStr"/>
+      <c r="AZ4" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="BA4" s="3" t="inlineStr"/>
+      <c r="BB4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane</t>
+          <t>98% confidence — extracted from DEBIT - NNELO</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+          <t>98% confidence — extracted from DEBIT - NNELO, p.2</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+          <t>98% confidence — extracted from DEBIT - NNELO, p.2</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
+          <t>98% confidence — extracted from DEBIT - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DEBIT - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DEBIT - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DEBIT - NNELO</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DEBIT - NNELO</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DEBIT - NNELO</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr"/>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
+      <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+          <t>98% confidence — extracted from DEBIT - NNELO, p.2</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="V5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
+          <t>98% confidence — extracted from DEBIT - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr"/>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="Y5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
+          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+        </is>
+      </c>
+      <c r="Y5" s="2" t="inlineStr"/>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
         </is>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="AC5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="AD5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
+          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+        </is>
+      </c>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
       <c r="AE5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="AF5" s="2" t="inlineStr"/>
-      <c r="AG5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="AH5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane</t>
-        </is>
-      </c>
-      <c r="AI5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="AJ5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="AK5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="AL5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
+          <t>80% confidence — extracted from DEBIT - NNELO, p.2 — ⚠ recommend recheck</t>
+        </is>
+      </c>
+      <c r="AF5" s="2" t="inlineStr">
+        <is>
+          <t>80% confidence — extracted from DEBIT - NNELO, p.2 — ⚠ recommend recheck</t>
+        </is>
+      </c>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
+      <c r="AK5" s="2" t="inlineStr"/>
+      <c r="AL5" s="2" t="inlineStr"/>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="AN5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="AO5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
-      <c r="AP5" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
-        </is>
-      </c>
+          <t>98% confidence — extracted from DEBIT - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="AN5" s="2" t="inlineStr"/>
+      <c r="AO5" s="2" t="inlineStr"/>
+      <c r="AP5" s="2" t="inlineStr"/>
+      <c r="AQ5" s="2" t="inlineStr"/>
+      <c r="AR5" s="2" t="inlineStr"/>
+      <c r="AS5" s="2" t="inlineStr"/>
+      <c r="AT5" s="2" t="inlineStr"/>
+      <c r="AU5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AW5" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DEBIT - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="AX5" s="2" t="inlineStr"/>
+      <c r="AY5" s="2" t="inlineStr"/>
+      <c r="AZ5" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from DEBIT - NNELO</t>
+        </is>
+      </c>
+      <c r="BA5" s="2" t="inlineStr"/>
+      <c r="BB5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>DIS - NNELO</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>DIS</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Disinvestment Form (Standard)</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>ADD - NNELO</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Additional Investment Form</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>NNelo Taunyane</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>11102222</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Unknown - Fund Name Not Extracted</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>99</v>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>Rejected</t>
-        </is>
-      </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>Validation failed: fund_name</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>NNELO TAUNYANE</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Bifm Pula Money Market Fund</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>1876545</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Money Market</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Captured</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr"/>
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="P6" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-02T17:10:12</t>
-        </is>
-      </c>
-      <c r="Q6" s="4" t="inlineStr">
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02T17:16:15</t>
+        </is>
+      </c>
+      <c r="R6" s="3" t="inlineStr">
         <is>
           <t>marvel.ai-local-poc</t>
         </is>
       </c>
-      <c r="R6" s="4" t="inlineStr"/>
-      <c r="S6" s="4" t="inlineStr">
+      <c r="S6" s="3" t="inlineStr"/>
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>71234567</t>
         </is>
       </c>
-      <c r="T6" s="4" t="inlineStr">
-        <is>
-          <t>nnelo@bifm.co.bw</t>
-        </is>
-      </c>
-      <c r="U6" s="4" t="inlineStr"/>
-      <c r="V6" s="4" t="inlineStr">
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>nneelo@bifm.co.bw</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="inlineStr"/>
+      <c r="W6" s="3" t="inlineStr">
         <is>
           <t>NNELO TAUNYANE</t>
         </is>
       </c>
-      <c r="W6" s="4" t="inlineStr">
+      <c r="X6" s="3" t="inlineStr">
         <is>
           <t>STANBIC</t>
         </is>
       </c>
-      <c r="X6" s="4" t="inlineStr">
-        <is>
-          <t>9060001231234</t>
-        </is>
-      </c>
-      <c r="Y6" s="4" t="inlineStr">
+      <c r="Y6" s="3" t="inlineStr"/>
+      <c r="Z6" s="3" t="inlineStr">
         <is>
           <t>FAIRGROUNDS</t>
         </is>
       </c>
-      <c r="Z6" s="4" t="inlineStr">
+      <c r="AA6" s="3" t="inlineStr">
         <is>
           <t>064967</t>
         </is>
       </c>
-      <c r="AA6" s="4" t="inlineStr">
+      <c r="AB6" s="3" t="inlineStr">
         <is>
           <t>Current</t>
         </is>
       </c>
-      <c r="AB6" s="4" t="inlineStr"/>
-      <c r="AC6" s="4" t="inlineStr"/>
-      <c r="AD6" s="4" t="inlineStr"/>
-      <c r="AE6" s="4" t="inlineStr"/>
-      <c r="AF6" s="4" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="AG6" s="4" t="inlineStr"/>
-      <c r="AH6" s="4" t="inlineStr"/>
-      <c r="AI6" s="4" t="inlineStr"/>
-      <c r="AJ6" s="4" t="inlineStr"/>
-      <c r="AK6" s="4" t="inlineStr"/>
-      <c r="AL6" s="4" t="inlineStr"/>
-      <c r="AM6" s="4" t="inlineStr"/>
-      <c r="AN6" s="4" t="inlineStr"/>
-      <c r="AO6" s="4" t="inlineStr"/>
-      <c r="AP6" s="4" t="inlineStr"/>
+      <c r="AC6" s="3" t="inlineStr"/>
+      <c r="AD6" s="3" t="inlineStr"/>
+      <c r="AE6" s="3" t="inlineStr"/>
+      <c r="AF6" s="3" t="inlineStr"/>
+      <c r="AG6" s="3" t="inlineStr"/>
+      <c r="AH6" s="3" t="inlineStr"/>
+      <c r="AI6" s="3" t="inlineStr"/>
+      <c r="AJ6" s="3" t="inlineStr"/>
+      <c r="AK6" s="3" t="inlineStr">
+        <is>
+          <t>Reinvest</t>
+        </is>
+      </c>
+      <c r="AL6" s="3" t="inlineStr"/>
+      <c r="AM6" s="3" t="inlineStr"/>
+      <c r="AN6" s="3" t="inlineStr"/>
+      <c r="AO6" s="3" t="inlineStr"/>
+      <c r="AP6" s="3" t="inlineStr"/>
+      <c r="AQ6" s="3" t="inlineStr"/>
+      <c r="AR6" s="3" t="inlineStr"/>
+      <c r="AS6" s="3" t="inlineStr">
+        <is>
+          <t>1000-00</t>
+        </is>
+      </c>
+      <c r="AT6" s="3" t="inlineStr"/>
+      <c r="AU6" s="3" t="inlineStr">
+        <is>
+          <t>Investor's bank account</t>
+        </is>
+      </c>
+      <c r="AV6" s="3" t="inlineStr"/>
+      <c r="AW6" s="3" t="inlineStr"/>
+      <c r="AX6" s="3" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="AY6" s="3" t="inlineStr"/>
+      <c r="AZ6" s="3" t="inlineStr"/>
+      <c r="BA6" s="3" t="inlineStr"/>
+      <c r="BB6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr"/>
       <c r="B7" s="2" t="inlineStr"/>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from DIS - NNELO</t>
+          <t>98% confidence — extracted from ADD - NNELO</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from ADD - NNELO, p.2</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
+          <t>98% confidence — extracted from ADD - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from ADD - NNELO, p.2</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from DIS - NNELO</t>
+          <t>98% confidence — extracted from ADD - NNELO, p.2</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from DIS - NNELO</t>
+          <t>98% confidence — extracted from ADD - NNELO</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from DIS - NNELO</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr"/>
+          <t>98% confidence — extracted from ADD - NNELO</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from ADD - NNELO</t>
+        </is>
+      </c>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
       <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr">
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from ADD - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from ADD - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr"/>
+      <c r="W7" s="2" t="inlineStr">
         <is>
           <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
         </is>
       </c>
-      <c r="T7" s="2" t="inlineStr">
+      <c r="X7" s="2" t="inlineStr">
         <is>
           <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
         </is>
       </c>
-      <c r="U7" s="2" t="inlineStr"/>
-      <c r="V7" s="2" t="inlineStr">
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr">
         <is>
           <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
         </is>
       </c>
-      <c r="W7" s="2" t="inlineStr">
+      <c r="AA7" s="2" t="inlineStr">
         <is>
           <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
         </is>
       </c>
-      <c r="X7" s="2" t="inlineStr">
+      <c r="AB7" s="2" t="inlineStr">
         <is>
           <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
         </is>
       </c>
-      <c r="Y7" s="2" t="inlineStr">
-        <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
-      <c r="Z7" s="2" t="inlineStr">
-        <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
-      <c r="AA7" s="2" t="inlineStr">
-        <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
-      <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr"/>
       <c r="AD7" s="2" t="inlineStr"/>
       <c r="AE7" s="2" t="inlineStr"/>
-      <c r="AF7" s="2" t="inlineStr">
-        <is>
-          <t>0% confidence — extracted from DIS - NNELO — ⚠ recommend recheck</t>
-        </is>
-      </c>
+      <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
       <c r="AI7" s="2" t="inlineStr"/>
       <c r="AJ7" s="2" t="inlineStr"/>
-      <c r="AK7" s="2" t="inlineStr"/>
+      <c r="AK7" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from ADD - NNELO, p.2</t>
+        </is>
+      </c>
       <c r="AL7" s="2" t="inlineStr"/>
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr"/>
       <c r="AO7" s="2" t="inlineStr"/>
       <c r="AP7" s="2" t="inlineStr"/>
+      <c r="AQ7" s="2" t="inlineStr"/>
+      <c r="AR7" s="2" t="inlineStr"/>
+      <c r="AS7" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from ADD - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="AT7" s="2" t="inlineStr"/>
+      <c r="AU7" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from ADD - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="AV7" s="2" t="inlineStr"/>
+      <c r="AW7" s="2" t="inlineStr"/>
+      <c r="AX7" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from ADD - NNELO, p.2</t>
+        </is>
+      </c>
+      <c r="AY7" s="2" t="inlineStr"/>
+      <c r="AZ7" s="2" t="inlineStr"/>
+      <c r="BA7" s="2" t="inlineStr"/>
+      <c r="BB7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>DEBIT - NNELO</t>
+          <t>GSGF - NNELO TAUNYANE</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>DEBIT</t>
+          <t>DIS_GSG</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Debit Order Form</t>
+          <t>Disinvestment Form (GSGF)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>381234567</t>
+          <t>381234321</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>NNelo Taunyane</t>
+          <t>NNELO TAUNYANE</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>11102222</t>
+          <t>111102222</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>Unknown - Fund Name Not Extracted</t>
-        </is>
-      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>BIFM Global Sustainable Growth Fund</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>99</v>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
+          <t>Non-Money Market (GSGF)</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Quarterly - 7th of last month of quarter</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>3</v>
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>Validation failed: instruction_type</t>
-        </is>
-      </c>
-      <c r="O8" s="4" t="inlineStr">
+          <t>Captured</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr"/>
+      <c r="P8" s="4" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="P8" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-02T17:10:12</t>
-        </is>
-      </c>
       <c r="Q8" s="4" t="inlineStr">
         <is>
+          <t>2026-07-02T17:16:15</t>
+        </is>
+      </c>
+      <c r="R8" s="4" t="inlineStr">
+        <is>
           <t>marvel.ai-local-poc</t>
         </is>
       </c>
-      <c r="R8" s="4" t="inlineStr"/>
-      <c r="S8" s="4" t="inlineStr">
+      <c r="S8" s="4" t="inlineStr"/>
+      <c r="T8" s="4" t="inlineStr">
         <is>
           <t>71234567</t>
         </is>
       </c>
-      <c r="T8" s="4" t="inlineStr">
+      <c r="U8" s="4" t="inlineStr">
         <is>
           <t>nnelo@bifm.co.bw</t>
         </is>
       </c>
-      <c r="U8" s="4" t="inlineStr"/>
-      <c r="V8" s="4" t="inlineStr">
+      <c r="V8" s="4" t="inlineStr"/>
+      <c r="W8" s="4" t="inlineStr">
         <is>
           <t>NNELO TAUNYANE</t>
         </is>
       </c>
-      <c r="W8" s="4" t="inlineStr">
+      <c r="X8" s="4" t="inlineStr">
         <is>
           <t>STANBIC</t>
         </is>
       </c>
-      <c r="X8" s="4" t="inlineStr">
-        <is>
-          <t>9060001231234</t>
-        </is>
-      </c>
       <c r="Y8" s="4" t="inlineStr">
         <is>
+          <t>906000123124</t>
+        </is>
+      </c>
+      <c r="Z8" s="4" t="inlineStr">
+        <is>
           <t>FAIRGROUNDS</t>
         </is>
       </c>
-      <c r="Z8" s="4" t="inlineStr">
+      <c r="AA8" s="4" t="inlineStr">
         <is>
           <t>064967</t>
         </is>
       </c>
-      <c r="AA8" s="4" t="inlineStr">
+      <c r="AB8" s="4" t="inlineStr">
         <is>
           <t>Current</t>
         </is>
       </c>
-      <c r="AB8" s="4" t="inlineStr"/>
       <c r="AC8" s="4" t="inlineStr"/>
-      <c r="AD8" s="4" t="inlineStr"/>
+      <c r="AD8" s="4" t="b">
+        <v>0</v>
+      </c>
       <c r="AE8" s="4" t="inlineStr"/>
       <c r="AF8" s="4" t="inlineStr"/>
       <c r="AG8" s="4" t="inlineStr"/>
-      <c r="AH8" s="4" t="inlineStr"/>
+      <c r="AH8" s="4" t="n">
+        <v>5000</v>
+      </c>
       <c r="AI8" s="4" t="inlineStr"/>
       <c r="AJ8" s="4" t="inlineStr"/>
       <c r="AK8" s="4" t="inlineStr"/>
-      <c r="AL8" s="4" t="inlineStr"/>
+      <c r="AL8" s="4" t="inlineStr">
+        <is>
+          <t>Partial Withdrawal</t>
+        </is>
+      </c>
       <c r="AM8" s="4" t="inlineStr"/>
       <c r="AN8" s="4" t="inlineStr"/>
       <c r="AO8" s="4" t="inlineStr"/>
       <c r="AP8" s="4" t="inlineStr"/>
+      <c r="AQ8" s="4" t="inlineStr"/>
+      <c r="AR8" s="4" t="inlineStr"/>
+      <c r="AS8" s="4" t="inlineStr"/>
+      <c r="AT8" s="4" t="inlineStr"/>
+      <c r="AU8" s="4" t="inlineStr"/>
+      <c r="AV8" s="4" t="inlineStr"/>
+      <c r="AW8" s="4" t="inlineStr"/>
+      <c r="AX8" s="4" t="inlineStr"/>
+      <c r="AY8" s="4" t="inlineStr"/>
+      <c r="AZ8" s="4" t="inlineStr"/>
+      <c r="BA8" s="4" t="inlineStr"/>
+      <c r="BB8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr"/>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from DEBIT - NNELO</t>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE, p.2</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE, p.2</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE, p.2</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from DEBIT - NNELO</t>
-        </is>
-      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from DEBIT - NNELO</t>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from DEBIT - NNELO</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr"/>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE</t>
+        </is>
+      </c>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr"/>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="inlineStr"/>
-      <c r="S9" s="2" t="inlineStr">
+      <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE, p.2</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE, p.2</t>
+        </is>
+      </c>
+      <c r="V9" s="2" t="inlineStr"/>
+      <c r="W9" s="2" t="inlineStr">
         <is>
           <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
         </is>
       </c>
-      <c r="T9" s="2" t="inlineStr">
-        <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
-      <c r="U9" s="2" t="inlineStr"/>
-      <c r="V9" s="2" t="inlineStr">
-        <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
-      <c r="W9" s="2" t="inlineStr">
-        <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE, p.2</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE, p.2</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE, p.2</t>
         </is>
       </c>
       <c r="AA9" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
-      <c r="AB9" s="2" t="inlineStr"/>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE, p.2</t>
+        </is>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE, p.2</t>
+        </is>
+      </c>
       <c r="AC9" s="2" t="inlineStr"/>
-      <c r="AD9" s="2" t="inlineStr"/>
+      <c r="AD9" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE, p.2</t>
+        </is>
+      </c>
       <c r="AE9" s="2" t="inlineStr"/>
       <c r="AF9" s="2" t="inlineStr"/>
       <c r="AG9" s="2" t="inlineStr"/>
-      <c r="AH9" s="2" t="inlineStr"/>
+      <c r="AH9" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE, p.2</t>
+        </is>
+      </c>
       <c r="AI9" s="2" t="inlineStr"/>
       <c r="AJ9" s="2" t="inlineStr"/>
       <c r="AK9" s="2" t="inlineStr"/>
-      <c r="AL9" s="2" t="inlineStr"/>
+      <c r="AL9" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from GSGF - NNELO TAUNYANE</t>
+        </is>
+      </c>
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr"/>
       <c r="AO9" s="2" t="inlineStr"/>
       <c r="AP9" s="2" t="inlineStr"/>
+      <c r="AQ9" s="2" t="inlineStr"/>
+      <c r="AR9" s="2" t="inlineStr"/>
+      <c r="AS9" s="2" t="inlineStr"/>
+      <c r="AT9" s="2" t="inlineStr"/>
+      <c r="AU9" s="2" t="inlineStr"/>
+      <c r="AV9" s="2" t="inlineStr"/>
+      <c r="AW9" s="2" t="inlineStr"/>
+      <c r="AX9" s="2" t="inlineStr"/>
+      <c r="AY9" s="2" t="inlineStr"/>
+      <c r="AZ9" s="2" t="inlineStr"/>
+      <c r="BA9" s="2" t="inlineStr"/>
+      <c r="BB9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Additional Investment Form</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>KYC - Nnelo Taunyane</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>KYC</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>KYC (Know Your Customer)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>NNelo Taunyane</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>Unknown - Fund Name Not Extracted</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>99</v>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="inlineStr">
-        <is>
-          <t>Rejected</t>
-        </is>
-      </c>
-      <c r="N10" s="4" t="inlineStr">
-        <is>
-          <t>Validation failed: fund_name, fund_number</t>
-        </is>
-      </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>11102222</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>01/02/2003</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Captured</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr"/>
+      <c r="P10" s="3" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="P10" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-02T17:10:12</t>
-        </is>
-      </c>
-      <c r="Q10" s="4" t="inlineStr">
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02T17:16:15</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
         <is>
           <t>marvel.ai-local-poc</t>
         </is>
       </c>
-      <c r="R10" s="4" t="inlineStr"/>
-      <c r="S10" s="4" t="inlineStr">
+      <c r="S10" s="3" t="inlineStr"/>
+      <c r="T10" s="3" t="inlineStr">
         <is>
           <t>71234567</t>
         </is>
       </c>
-      <c r="T10" s="4" t="inlineStr">
+      <c r="U10" s="3" t="inlineStr">
         <is>
           <t>nnelo@bifm.co.bw</t>
         </is>
       </c>
-      <c r="U10" s="4" t="inlineStr"/>
-      <c r="V10" s="4" t="inlineStr">
+      <c r="V10" s="3" t="inlineStr">
+        <is>
+          <t>MOTSWANA</t>
+        </is>
+      </c>
+      <c r="W10" s="3" t="inlineStr">
         <is>
           <t>NNELO TAUNYANE</t>
         </is>
       </c>
-      <c r="W10" s="4" t="inlineStr">
+      <c r="X10" s="3" t="inlineStr">
         <is>
           <t>STANBIC</t>
         </is>
       </c>
-      <c r="X10" s="4" t="inlineStr">
+      <c r="Y10" s="3" t="inlineStr">
         <is>
           <t>9060001231234</t>
         </is>
       </c>
-      <c r="Y10" s="4" t="inlineStr">
+      <c r="Z10" s="3" t="inlineStr">
         <is>
           <t>FAIRGROUNDS</t>
         </is>
       </c>
-      <c r="Z10" s="4" t="inlineStr">
+      <c r="AA10" s="3" t="inlineStr">
         <is>
           <t>064967</t>
         </is>
       </c>
-      <c r="AA10" s="4" t="inlineStr">
+      <c r="AB10" s="3" t="inlineStr">
         <is>
           <t>Current</t>
         </is>
       </c>
-      <c r="AB10" s="4" t="inlineStr"/>
-      <c r="AC10" s="4" t="inlineStr"/>
-      <c r="AD10" s="4" t="inlineStr"/>
-      <c r="AE10" s="4" t="inlineStr"/>
-      <c r="AF10" s="4" t="inlineStr"/>
-      <c r="AG10" s="4" t="inlineStr"/>
-      <c r="AH10" s="4" t="inlineStr"/>
-      <c r="AI10" s="4" t="inlineStr"/>
-      <c r="AJ10" s="4" t="inlineStr"/>
-      <c r="AK10" s="4" t="inlineStr"/>
-      <c r="AL10" s="4" t="inlineStr"/>
-      <c r="AM10" s="4" t="inlineStr"/>
-      <c r="AN10" s="4" t="inlineStr"/>
-      <c r="AO10" s="4" t="inlineStr"/>
-      <c r="AP10" s="4" t="inlineStr"/>
+      <c r="AC10" s="3" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="AD10" s="3" t="inlineStr"/>
+      <c r="AE10" s="3" t="inlineStr"/>
+      <c r="AF10" s="3" t="inlineStr"/>
+      <c r="AG10" s="3" t="inlineStr">
+        <is>
+          <t>BOTSWANA</t>
+        </is>
+      </c>
+      <c r="AH10" s="3" t="inlineStr"/>
+      <c r="AI10" s="3" t="inlineStr">
+        <is>
+          <t>BIFM UNIT TRUSTS</t>
+        </is>
+      </c>
+      <c r="AJ10" s="3" t="inlineStr">
+        <is>
+          <t>NNELO TAUNYANE</t>
+        </is>
+      </c>
+      <c r="AK10" s="3" t="inlineStr"/>
+      <c r="AL10" s="3" t="inlineStr"/>
+      <c r="AM10" s="3" t="inlineStr"/>
+      <c r="AN10" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO10" s="3" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="AP10" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ10" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AR10" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS10" s="3" t="inlineStr"/>
+      <c r="AT10" s="3" t="inlineStr">
+        <is>
+          <t>INTERN</t>
+        </is>
+      </c>
+      <c r="AU10" s="3" t="inlineStr"/>
+      <c r="AV10" s="3" t="inlineStr">
+        <is>
+          <t>PLOT 1234 GABORONE</t>
+        </is>
+      </c>
+      <c r="AW10" s="3" t="inlineStr"/>
+      <c r="AX10" s="3" t="inlineStr"/>
+      <c r="AY10" s="3" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="AZ10" s="3" t="inlineStr"/>
+      <c r="BA10" s="3" t="inlineStr">
+        <is>
+          <t>Ms</t>
+        </is>
+      </c>
+      <c r="BB10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr"/>
       <c r="B11" s="2" t="inlineStr"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>98% confidence — extracted from ADD - NNELO</t>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>98% confidence — extracted from ADD - NNELO</t>
-        </is>
-      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr"/>
@@ -2287,62 +2516,134 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
       <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="2" t="inlineStr">
-        <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
+      <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
-      <c r="U11" s="2" t="inlineStr"/>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
         </is>
       </c>
       <c r="W11" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
         </is>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
         </is>
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
         </is>
       </c>
       <c r="AA11" s="2" t="inlineStr">
         <is>
-          <t>85% confidence — backfilled from KYC - Nnelo Taunyane — ⚠ recommend recheck</t>
-        </is>
-      </c>
-      <c r="AB11" s="2" t="inlineStr"/>
-      <c r="AC11" s="2" t="inlineStr"/>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
       <c r="AD11" s="2" t="inlineStr"/>
       <c r="AE11" s="2" t="inlineStr"/>
       <c r="AF11" s="2" t="inlineStr"/>
-      <c r="AG11" s="2" t="inlineStr"/>
+      <c r="AG11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
       <c r="AH11" s="2" t="inlineStr"/>
-      <c r="AI11" s="2" t="inlineStr"/>
-      <c r="AJ11" s="2" t="inlineStr"/>
+      <c r="AI11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="AJ11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
       <c r="AK11" s="2" t="inlineStr"/>
       <c r="AL11" s="2" t="inlineStr"/>
       <c r="AM11" s="2" t="inlineStr"/>
-      <c r="AN11" s="2" t="inlineStr"/>
-      <c r="AO11" s="2" t="inlineStr"/>
-      <c r="AP11" s="2" t="inlineStr"/>
+      <c r="AN11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="AO11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane</t>
+        </is>
+      </c>
+      <c r="AP11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="AQ11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="AR11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="AS11" s="2" t="inlineStr"/>
+      <c r="AT11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="AU11" s="2" t="inlineStr"/>
+      <c r="AV11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="AW11" s="2" t="inlineStr"/>
+      <c r="AX11" s="2" t="inlineStr"/>
+      <c r="AY11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="AZ11" s="2" t="inlineStr"/>
+      <c r="BA11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
+      <c r="BB11" s="2" t="inlineStr">
+        <is>
+          <t>98% confidence — extracted from KYC - Nnelo Taunyane, p.1</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2403,14 +2704,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
@@ -2453,33 +2754,33 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>KYC - Nnelo Taunyane</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>KYC</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="E2" s="5" t="n"/>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Gender derivation not applicable for this ID type</t>
         </is>
@@ -2519,338 +2820,334 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>KYC - Nnelo Taunyane</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>KYC</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>date_of_birth</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>01/02/2003</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>KYC - Nnelo Taunyane</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>KYC</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>nnelo@bifm.co.bw</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>KYC - Nnelo Taunyane</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>KYC</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>contact_number</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>71234567</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>KYC - Nnelo Taunyane</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>KYC</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>branch_code</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>064967</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>KYC - Nnelo Taunyane</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>KYC</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>kyc_completeness_flag</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>381234321</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>GSGF - NNELO TAUNYANE</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>DIS_GSG</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>nnelo@bifm.co.bw</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>381234321</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>GSGF - NNELO TAUNYANE</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>DIS_GSG</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>contact_number</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>71234567</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>381234321</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>GSGF - NNELO TAUNYANE</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>DIS_GSG</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>branch_code</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>064967</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>381234321</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>GSGF - NNELO TAUNYANE</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>DIS_GSG</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>fund_category</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Non-Money Market (GSGF)</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>381234321</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>GSGF - NNELO TAUNYANE</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>DIS_GSG</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>instruction_mode</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Could not determine instruction mode - no closure tick, percentage, or withdrawal/deposit amount was found</t>
-        </is>
-      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Partial Withdrawal</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -2870,226 +3167,222 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>fund_name</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="n"/>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>nnelo@bifm.co.bw</t>
+        </is>
+      </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Mandatory field missing</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>DIS - NNELO</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>DIS</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>contact_number</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>71234567</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>DIS - NNELO</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>branch_code</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>064967</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>DIS - NNELO</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>fund_number</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>9876543</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Expected 8 or 9 digits, got 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>DIS - NNELO</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>fund_category</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Money Market</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>DIS - NNELO</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>instruction_mode</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Partial Withdrawal</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>DEBIT - NNELO</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>DEBIT</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>nnelo@bifm.co.bw</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>taunyane@bifm.co.bw</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>DIS - NNELO</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>DIS</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>contact_number</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>71234567</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>DIS - NNELO</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>DIS</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>branch_code</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>064967</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>DIS - NNELO</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>DIS</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>fund_number</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Field is blank</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>DIS - NNELO</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>DIS</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>fund_category</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>Unknown - Fund Name Not Extracted</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Fund category could not be determined - fund name unclear</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>DIS - NNELO</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>DIS</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>instruction_mode</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Could not determine instruction mode - no closure tick, percentage, or withdrawal/deposit amount was found</t>
-        </is>
-      </c>
+      <c r="G20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -3109,189 +3402,189 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>instruction_type</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n"/>
+          <t>contact_number</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>71234567</t>
+        </is>
+      </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Mandatory field missing</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>DEBIT - NNELO</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>DEBIT</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>branch_code</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>064967</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>DEBIT - NNELO</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>DEBIT</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>fund_number</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>9876543</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Expected 8 or 9 digits, got 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>DEBIT - NNELO</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>DEBIT</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>fund_category</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Money Market</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>381234567</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>ADD - NNELO</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>nnelo@bifm.co.bw</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>nneelo@bifm.co.bw</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>DEBIT - NNELO</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>DEBIT</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>ADD - NNELO</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>contact_number</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>71234567</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>DEBIT - NNELO</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>DEBIT</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>branch_code</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>064967</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>DEBIT - NNELO</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>DEBIT</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>fund_number</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Field is blank</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>DEBIT - NNELO</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>DEBIT</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>fund_category</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>Unknown - Fund Name Not Extracted</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Fund category could not be determined - fund name unclear</t>
-        </is>
-      </c>
+      <c r="G26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -3311,222 +3604,90 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>fund_name</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="n"/>
+          <t>branch_code</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>064967</t>
+        </is>
+      </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>Mandatory field missing</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>ADD - NNELO</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>ADD</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>fund_number</t>
         </is>
       </c>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>Mandatory field missing</t>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>1876545</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Expected 8 or 9 digits, got 7</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>381234567</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>ADD - NNELO</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>ADD</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>nnelo@bifm.co.bw</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>fund_category</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Money Market</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>contact_number</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>71234567</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>branch_code</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>064967</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>fund_number</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="n"/>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Field is blank</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>381234567</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>ADD - NNELO</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>fund_category</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Unknown - Fund Name Not Extracted</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>Fund category could not be determined - fund name unclear</t>
-        </is>
-      </c>
+      <c r="G29" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3549,7 +3710,7 @@
     <col width="27" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="43" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
@@ -3633,7 +3794,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:11:20</t>
+          <t>2026-07-02T17:18:22</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3643,7 +3804,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KYC_381234567_TAUNYANE_20260702_1_2_3.pdf</t>
+          <t>KYC_381234567_TAUNYANE_20260702_1_2_3_4.pdf</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -3672,12 +3833,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:10:12</t>
+          <t>2026-07-02T17:16:15</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\KYC_381234567_TAUNYANE_20260702_1_2_3.pdf</t>
+          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\KYC_381234567_TAUNYANE_20260702_1_2_3_4.pdf</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -3695,7 +3856,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-02T17:11:20</t>
+          <t>2026-07-02T17:18:22</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3705,7 +3866,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DIS_GSG_381234567_TAUNYANE_20260702_1_2_3.pdf</t>
+          <t>DIS_GSG_381234321_TAUNYANE_20260702.pdf</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -3718,7 +3879,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -3734,12 +3895,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-02T17:10:12</t>
+          <t>2026-07-02T17:16:15</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\DIS_GSG_381234567_TAUNYANE_20260702_1_2_3.pdf</t>
+          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\DIS_GSG_381234321_TAUNYANE_20260702.pdf</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -3757,7 +3918,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-02T17:11:20</t>
+          <t>2026-07-02T17:18:22</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3767,7 +3928,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DIS_381234567_TAUNYANE_20260702_VALIDATIONFAILEDFUND_NAME_1_2_3.pdf</t>
+          <t>DIS_381234567_TAUNYANE_20260702.pdf</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -3776,23 +3937,19 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Rejected</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Validation failed: fund_name</t>
-        </is>
-      </c>
+          <t>Captured</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>Email</t>
@@ -3800,12 +3957,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-02T17:10:12</t>
+          <t>2026-07-02T17:16:15</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\Rejected\DIS_381234567_TAUNYANE_20260702_VALIDATIONFAILEDFUND_NAME_1_2_3.pdf</t>
+          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\MoneyMarket\Captured\DIS_381234567_TAUNYANE_20260702.pdf</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -3823,7 +3980,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:11:20</t>
+          <t>2026-07-02T17:18:22</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3833,7 +3990,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DEBIT_381234567_TAUNYANE_20260702_VALIDATIONFAILEDINSTRUCTION_TYPE_1_2_3.pdf</t>
+          <t>DEBIT_381234567_TAUNYANE_20260702.pdf</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -3846,19 +4003,15 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Rejected</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Validation failed: instruction_type</t>
-        </is>
-      </c>
+          <t>Captured</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>Email</t>
@@ -3866,12 +4019,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:10:12</t>
+          <t>2026-07-02T17:16:15</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\Rejected\DEBIT_381234567_TAUNYANE_20260702_VALIDATIONFAILEDINSTRUCTION_TYPE_1_2_3.pdf</t>
+          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\MoneyMarket\Captured\DEBIT_381234567_TAUNYANE_20260702.pdf</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -3889,7 +4042,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-02T17:11:20</t>
+          <t>2026-07-02T17:18:22</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3899,7 +4052,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ADD_381234567_TAUNYANE_20260702_VALIDATIONFAILEDFUND_NAMEFUND_NUMBER_1_2_3.pdf</t>
+          <t>ADD_381234567_TAUNYANE_20260702.pdf</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -3912,19 +4065,15 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Rejected</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Validation failed: fund_name, fund_number</t>
-        </is>
-      </c>
+          <t>Captured</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>Email</t>
@@ -3932,12 +4081,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-02T17:10:12</t>
+          <t>2026-07-02T17:16:15</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\NonMoneyMarket\Captured\Rejected\ADD_381234567_TAUNYANE_20260702_VALIDATIONFAILEDFUND_NAMEFUND_NUMBER_1_2_3.pdf</t>
+          <t>C:\Users\dhruv\OneDrive\Documents\GitHub\BIFMPoC\output\filed_documents\2026\07-July\02\MoneyMarket\Captured\ADD_381234567_TAUNYANE_20260702.pdf</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">

</xml_diff>